<commit_message>
data: Todas - Relatorio de Pendencias - 19-06-26 1607.xlsx
</commit_message>
<xml_diff>
--- a/data/coordenadores/Coordenadores (SP-RJ-Santos).xlsx
+++ b/data/coordenadores/Coordenadores (SP-RJ-Santos).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\GERÊNCIA\Gerencia Operacional\CTR\Juan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A913EE7-9821-411D-908D-3CDF5817F2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0EB4B3-93CA-413A-BAFF-474589CD6B45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="547">
   <si>
     <t>ADRIANO DE BARROS DOS SANTOS</t>
   </si>
@@ -596,9 +596,6 @@
     <t>Heloise Venancio</t>
   </si>
   <si>
-    <t>Idna Sousa</t>
-  </si>
-  <si>
     <t>IGOR LEONARDO VALEZI</t>
   </si>
   <si>
@@ -863,9 +860,6 @@
     <t>Laisa Rocha</t>
   </si>
   <si>
-    <t>Larice Souza</t>
-  </si>
-  <si>
     <t>LARISSA FERNANDES FELIX</t>
   </si>
   <si>
@@ -1676,16 +1670,10 @@
     <t>Nome Completo</t>
   </si>
   <si>
-    <t>Walace Gonçalves | Maicon Costa</t>
-  </si>
-  <si>
-    <t>Karina Oliveira | Liliane Costa</t>
-  </si>
-  <si>
-    <t>Julio Santos | Jessica Benjamin</t>
-  </si>
-  <si>
-    <t>Erika Santana | Isabella Nascimento</t>
+    <t>Luiz Ferreira</t>
+  </si>
+  <si>
+    <t>Claudineia Rodrigues</t>
   </si>
 </sst>
 </file>
@@ -1693,8 +1681,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="166" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -1720,7 +1708,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1735,6 +1723,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1765,22 +1759,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="Comma 2" xfId="6" xr:uid="{15B735D9-634A-47C1-8273-A48121050E52}"/>
@@ -1799,6 +1794,20 @@
     <cellStyle name="Vírgula 2" xfId="3" xr:uid="{44D8D12C-B8F2-4B7E-8E60-FE31C4C19D54}"/>
   </cellStyles>
   <dxfs count="3">
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1832,20 +1841,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1860,11 +1855,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F6AE6F53-2DB4-44BA-B797-40D5F442D5D6}" name="Tabela1" displayName="Tabela1" ref="A1:D259" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
-  <autoFilter ref="A1:D259" xr:uid="{F6AE6F53-2DB4-44BA-B797-40D5F442D5D6}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D259">
-    <sortCondition ref="C1:C259"/>
-  </sortState>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F6AE6F53-2DB4-44BA-B797-40D5F442D5D6}" name="Tabela1" displayName="Tabela1" ref="A1:D260" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A1:D260" xr:uid="{F6AE6F53-2DB4-44BA-B797-40D5F442D5D6}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF96588-4F5A-4B5F-95C5-9DAEC50CBCA7}" name="Nome Completo"/>
     <tableColumn id="2" xr3:uid="{5E6A984F-4C15-4C90-8F36-7C9BBA83F991}" name="Nome de Exibição"/>
@@ -2195,7 +2187,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D259"/>
+  <dimension ref="A1:D260"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.85546875" customWidth="1"/>
@@ -2206,16 +2198,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2229,35 +2221,35 @@
         <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B3" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C3" t="s">
         <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="B4" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C4" t="s">
         <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2271,7 +2263,7 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -2285,7 +2277,7 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2299,7 +2291,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -2313,7 +2305,7 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -2327,7 +2319,7 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2341,7 +2333,7 @@
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -2355,7 +2347,7 @@
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -2369,7 +2361,7 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2383,217 +2375,217 @@
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>193</v>
+      </c>
+      <c r="B14" t="s">
         <v>194</v>
-      </c>
-      <c r="B14" t="s">
-        <v>195</v>
       </c>
       <c r="C14" t="s">
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>273</v>
+      </c>
+      <c r="B15" t="s">
         <v>274</v>
-      </c>
-      <c r="B15" t="s">
-        <v>275</v>
       </c>
       <c r="C15" t="s">
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B16" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C16" t="s">
         <v>2</v>
       </c>
       <c r="D16" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B17" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
       <c r="D17" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B18" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C18" t="s">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B19" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C19" t="s">
         <v>2</v>
       </c>
       <c r="D19" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B20" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C20" t="s">
         <v>2</v>
       </c>
       <c r="D20" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B21" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C21" t="s">
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B22" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C22" t="s">
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B23" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C23" t="s">
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B24" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C24" t="s">
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B25" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C25" t="s">
         <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B26" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C26" t="s">
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>550</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="B27" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C27" t="s">
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B28" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C28" t="s">
         <v>2</v>
       </c>
       <c r="D28" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2607,35 +2599,35 @@
         <v>2</v>
       </c>
       <c r="D29" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B30" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="C30" t="s">
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B31" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C31" t="s">
         <v>2</v>
       </c>
       <c r="D31" t="s">
-        <v>550</v>
+        <v>136</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -2696,10 +2688,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>199</v>
+      </c>
+      <c r="B36" t="s">
         <v>200</v>
-      </c>
-      <c r="B36" t="s">
-        <v>201</v>
       </c>
       <c r="C36" t="s">
         <v>8</v>
@@ -2710,10 +2702,10 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B37" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C37" t="s">
         <v>8</v>
@@ -2724,10 +2716,10 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B38" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C38" t="s">
         <v>8</v>
@@ -2738,10 +2730,10 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B39" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C39" t="s">
         <v>8</v>
@@ -2752,10 +2744,10 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B40" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C40" t="s">
         <v>8</v>
@@ -2864,10 +2856,10 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B48" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C48" t="s">
         <v>8</v>
@@ -2892,10 +2884,10 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>191</v>
+      </c>
+      <c r="B50" t="s">
         <v>192</v>
-      </c>
-      <c r="B50" t="s">
-        <v>193</v>
       </c>
       <c r="C50" t="s">
         <v>8</v>
@@ -2906,10 +2898,10 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B51" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C51" t="s">
         <v>8</v>
@@ -2920,10 +2912,10 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B52" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C52" t="s">
         <v>8</v>
@@ -2934,10 +2926,10 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="B53" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="C53" t="s">
         <v>8</v>
@@ -2957,7 +2949,7 @@
         <v>8</v>
       </c>
       <c r="D54" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -2971,7 +2963,7 @@
         <v>8</v>
       </c>
       <c r="D55" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2985,7 +2977,7 @@
         <v>8</v>
       </c>
       <c r="D56" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -2999,7 +2991,7 @@
         <v>8</v>
       </c>
       <c r="D57" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -3013,63 +3005,63 @@
         <v>8</v>
       </c>
       <c r="D58" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B59" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C59" t="s">
         <v>8</v>
       </c>
       <c r="D59" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B60" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C60" t="s">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B61" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C61" t="s">
         <v>8</v>
       </c>
       <c r="D61" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B62" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="C62" t="s">
         <v>8</v>
       </c>
       <c r="D62" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -3083,63 +3075,63 @@
         <v>8</v>
       </c>
       <c r="D63" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>207</v>
+      </c>
+      <c r="B64" t="s">
         <v>208</v>
-      </c>
-      <c r="B64" t="s">
-        <v>209</v>
       </c>
       <c r="C64" t="s">
         <v>8</v>
       </c>
       <c r="D64" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B65" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C65" t="s">
         <v>8</v>
       </c>
       <c r="D65" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B66" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C66" t="s">
         <v>8</v>
       </c>
       <c r="D66" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B67" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C67" t="s">
         <v>8</v>
       </c>
       <c r="D67" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -3153,35 +3145,35 @@
         <v>8</v>
       </c>
       <c r="D68" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B69" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C69" t="s">
         <v>8</v>
       </c>
       <c r="D69" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B70" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C70" t="s">
         <v>8</v>
       </c>
       <c r="D70" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -3195,7 +3187,7 @@
         <v>8</v>
       </c>
       <c r="D71" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -3270,10 +3262,10 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>201</v>
+      </c>
+      <c r="B77" t="s">
         <v>202</v>
-      </c>
-      <c r="B77" t="s">
-        <v>203</v>
       </c>
       <c r="C77" t="s">
         <v>13</v>
@@ -3284,10 +3276,10 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B78" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C78" t="s">
         <v>13</v>
@@ -3298,10 +3290,10 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B79" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C79" t="s">
         <v>13</v>
@@ -3312,10 +3304,10 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B80" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="C80" t="s">
         <v>13</v>
@@ -3326,10 +3318,10 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B81" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C81" t="s">
         <v>13</v>
@@ -3340,10 +3332,10 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B82" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C82" t="s">
         <v>13</v>
@@ -3354,10 +3346,10 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B83" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C83" t="s">
         <v>13</v>
@@ -3368,10 +3360,10 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B84" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="C84" t="s">
         <v>13</v>
@@ -3382,10 +3374,10 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="B85" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C85" t="s">
         <v>13</v>
@@ -3396,10 +3388,10 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="B86" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="C86" t="s">
         <v>13</v>
@@ -3480,10 +3472,10 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>203</v>
+      </c>
+      <c r="B92" t="s">
         <v>204</v>
-      </c>
-      <c r="B92" t="s">
-        <v>205</v>
       </c>
       <c r="C92" t="s">
         <v>13</v>
@@ -3494,10 +3486,10 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>222</v>
+      </c>
+      <c r="B93" t="s">
         <v>223</v>
-      </c>
-      <c r="B93" t="s">
-        <v>224</v>
       </c>
       <c r="C93" t="s">
         <v>13</v>
@@ -3508,10 +3500,10 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>228</v>
+      </c>
+      <c r="B94" t="s">
         <v>229</v>
-      </c>
-      <c r="B94" t="s">
-        <v>230</v>
       </c>
       <c r="C94" t="s">
         <v>13</v>
@@ -3522,10 +3514,10 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B95" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C95" t="s">
         <v>13</v>
@@ -3536,10 +3528,10 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B96" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C96" t="s">
         <v>13</v>
@@ -3550,10 +3542,10 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B97" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C97" t="s">
         <v>13</v>
@@ -3564,10 +3556,10 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B98" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C98" t="s">
         <v>13</v>
@@ -3578,10 +3570,10 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B99" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C99" t="s">
         <v>13</v>
@@ -3592,10 +3584,10 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B100" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="C100" t="s">
         <v>13</v>
@@ -3606,10 +3598,10 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B101" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C101" t="s">
         <v>13</v>
@@ -3629,7 +3621,7 @@
         <v>13</v>
       </c>
       <c r="D102" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -3643,49 +3635,49 @@
         <v>13</v>
       </c>
       <c r="D103" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
+        <v>259</v>
+      </c>
+      <c r="B104" t="s">
         <v>260</v>
-      </c>
-      <c r="B104" t="s">
-        <v>261</v>
       </c>
       <c r="C104" t="s">
         <v>13</v>
       </c>
       <c r="D104" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B105" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C105" t="s">
         <v>13</v>
       </c>
       <c r="D105" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B106" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C106" t="s">
         <v>13</v>
       </c>
       <c r="D106" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -3699,7 +3691,7 @@
         <v>13</v>
       </c>
       <c r="D107" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -3713,7 +3705,7 @@
         <v>13</v>
       </c>
       <c r="D108" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -3727,105 +3719,105 @@
         <v>13</v>
       </c>
       <c r="D109" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
+        <v>212</v>
+      </c>
+      <c r="B110" t="s">
         <v>213</v>
-      </c>
-      <c r="B110" t="s">
-        <v>214</v>
       </c>
       <c r="C110" t="s">
         <v>13</v>
       </c>
       <c r="D110" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>250</v>
+      </c>
+      <c r="B111" t="s">
         <v>251</v>
-      </c>
-      <c r="B111" t="s">
-        <v>252</v>
       </c>
       <c r="C111" t="s">
         <v>13</v>
       </c>
       <c r="D111" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
+        <v>261</v>
+      </c>
+      <c r="B112" t="s">
         <v>262</v>
-      </c>
-      <c r="B112" t="s">
-        <v>263</v>
       </c>
       <c r="C112" t="s">
         <v>13</v>
       </c>
       <c r="D112" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B113" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C113" t="s">
         <v>13</v>
       </c>
       <c r="D113" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B114" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C114" t="s">
         <v>13</v>
       </c>
       <c r="D114" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B115" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C115" t="s">
         <v>13</v>
       </c>
       <c r="D115" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B116" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C116" t="s">
         <v>13</v>
       </c>
       <c r="D116" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -3839,7 +3831,7 @@
         <v>36</v>
       </c>
       <c r="D117" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -3853,7 +3845,7 @@
         <v>36</v>
       </c>
       <c r="D118" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -3867,7 +3859,7 @@
         <v>36</v>
       </c>
       <c r="D119" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -3881,7 +3873,7 @@
         <v>36</v>
       </c>
       <c r="D120" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -3895,49 +3887,49 @@
         <v>36</v>
       </c>
       <c r="D121" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
+        <v>230</v>
+      </c>
+      <c r="B122" t="s">
         <v>231</v>
-      </c>
-      <c r="B122" t="s">
-        <v>232</v>
       </c>
       <c r="C122" t="s">
         <v>36</v>
       </c>
       <c r="D122" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
+        <v>271</v>
+      </c>
+      <c r="B123" t="s">
         <v>272</v>
-      </c>
-      <c r="B123" t="s">
-        <v>273</v>
       </c>
       <c r="C123" t="s">
         <v>36</v>
       </c>
       <c r="D123" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B124" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C124" t="s">
         <v>36</v>
       </c>
       <c r="D124" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
@@ -3951,7 +3943,7 @@
         <v>36</v>
       </c>
       <c r="D125" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
@@ -3965,203 +3957,203 @@
         <v>36</v>
       </c>
       <c r="D126" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B127" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C127" t="s">
         <v>36</v>
       </c>
       <c r="D127" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B128" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C128" t="s">
         <v>36</v>
       </c>
       <c r="D128" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B129" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C129" t="s">
         <v>36</v>
       </c>
       <c r="D129" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="B130" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C130" t="s">
         <v>36</v>
       </c>
       <c r="D130" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="B131" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C131" t="s">
         <v>36</v>
       </c>
       <c r="D131" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B132" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="C132" t="s">
         <v>36</v>
       </c>
       <c r="D132" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B133" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C133" t="s">
         <v>36</v>
       </c>
       <c r="D133" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B134" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C134" t="s">
         <v>36</v>
       </c>
       <c r="D134" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B135" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C135" t="s">
         <v>36</v>
       </c>
       <c r="D135" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B136" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C136" t="s">
         <v>36</v>
       </c>
       <c r="D136" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B137" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="C137" t="s">
         <v>36</v>
       </c>
       <c r="D137" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B138" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C138" t="s">
         <v>36</v>
       </c>
       <c r="D138" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B139" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C139" t="s">
         <v>36</v>
       </c>
       <c r="D139" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B140" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C140" t="s">
         <v>36</v>
       </c>
       <c r="D140" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
@@ -4175,63 +4167,63 @@
         <v>5</v>
       </c>
       <c r="D141" t="s">
-        <v>187</v>
+        <v>546</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
+        <v>197</v>
+      </c>
+      <c r="B142" t="s">
         <v>198</v>
-      </c>
-      <c r="B142" t="s">
-        <v>199</v>
       </c>
       <c r="C142" t="s">
         <v>5</v>
       </c>
       <c r="D142" t="s">
-        <v>187</v>
+        <v>546</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>414</v>
-      </c>
-      <c r="B143" t="s">
-        <v>415</v>
-      </c>
-      <c r="C143" t="s">
+      <c r="A143" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="C143" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D143" t="s">
-        <v>187</v>
+      <c r="D143" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
-        <v>472</v>
-      </c>
-      <c r="B144" t="s">
-        <v>473</v>
-      </c>
-      <c r="C144" t="s">
+      <c r="A144" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="C144" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D144" t="s">
-        <v>187</v>
+      <c r="D144" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B145" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C145" t="s">
         <v>5</v>
       </c>
       <c r="D145" t="s">
-        <v>187</v>
+        <v>546</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
@@ -4245,7 +4237,7 @@
         <v>5</v>
       </c>
       <c r="D146" t="s">
-        <v>276</v>
+        <v>494</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
@@ -4259,133 +4251,133 @@
         <v>5</v>
       </c>
       <c r="D147" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
+        <v>187</v>
+      </c>
+      <c r="B148" t="s">
         <v>188</v>
-      </c>
-      <c r="B148" t="s">
-        <v>189</v>
       </c>
       <c r="C148" t="s">
         <v>5</v>
       </c>
       <c r="D148" t="s">
-        <v>276</v>
+        <v>432</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
+        <v>226</v>
+      </c>
+      <c r="B149" t="s">
         <v>227</v>
-      </c>
-      <c r="B149" t="s">
-        <v>228</v>
       </c>
       <c r="C149" t="s">
         <v>5</v>
       </c>
       <c r="D149" t="s">
-        <v>276</v>
+        <v>432</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
+        <v>234</v>
+      </c>
+      <c r="B150" t="s">
         <v>235</v>
-      </c>
-      <c r="B150" t="s">
-        <v>236</v>
       </c>
       <c r="C150" t="s">
         <v>5</v>
       </c>
       <c r="D150" t="s">
-        <v>276</v>
+        <v>432</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
+        <v>242</v>
+      </c>
+      <c r="B151" t="s">
         <v>243</v>
-      </c>
-      <c r="B151" t="s">
-        <v>244</v>
       </c>
       <c r="C151" t="s">
         <v>5</v>
       </c>
       <c r="D151" t="s">
-        <v>276</v>
+        <v>432</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
+        <v>244</v>
+      </c>
+      <c r="B152" t="s">
         <v>245</v>
-      </c>
-      <c r="B152" t="s">
-        <v>246</v>
       </c>
       <c r="C152" t="s">
         <v>5</v>
       </c>
       <c r="D152" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B153" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C153" t="s">
         <v>5</v>
       </c>
       <c r="D153" t="s">
-        <v>276</v>
+        <v>432</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B154" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C154" t="s">
         <v>5</v>
       </c>
       <c r="D154" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B155" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="C155" t="s">
         <v>5</v>
       </c>
       <c r="D155" t="s">
-        <v>276</v>
+        <v>432</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B156" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C156" t="s">
         <v>5</v>
       </c>
       <c r="D156" t="s">
-        <v>276</v>
+        <v>432</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
@@ -4399,7 +4391,7 @@
         <v>5</v>
       </c>
       <c r="D157" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
@@ -4413,7 +4405,7 @@
         <v>5</v>
       </c>
       <c r="D158" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
@@ -4427,7 +4419,7 @@
         <v>5</v>
       </c>
       <c r="D159" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
@@ -4441,91 +4433,91 @@
         <v>5</v>
       </c>
       <c r="D160" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
+        <v>224</v>
+      </c>
+      <c r="B161" t="s">
         <v>225</v>
-      </c>
-      <c r="B161" t="s">
-        <v>226</v>
       </c>
       <c r="C161" t="s">
         <v>5</v>
       </c>
       <c r="D161" t="s">
-        <v>301</v>
+        <v>432</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
+        <v>236</v>
+      </c>
+      <c r="B162" t="s">
         <v>237</v>
-      </c>
-      <c r="B162" t="s">
-        <v>238</v>
       </c>
       <c r="C162" t="s">
         <v>5</v>
       </c>
       <c r="D162" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
+      <c r="A163" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B163" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="B163" t="s">
-        <v>240</v>
-      </c>
-      <c r="C163" t="s">
+      <c r="C163" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D163" t="s">
-        <v>301</v>
+      <c r="D163" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B164" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C164" t="s">
         <v>5</v>
       </c>
       <c r="D164" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
-        <v>382</v>
-      </c>
-      <c r="B165" t="s">
-        <v>383</v>
-      </c>
-      <c r="C165" t="s">
+      <c r="A165" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="B165" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="C165" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D165" t="s">
-        <v>301</v>
+      <c r="D165" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
+      <c r="A166" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B166" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C166" t="s">
+      <c r="C166" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D166" t="s">
-        <v>434</v>
+      <c r="D166" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
@@ -4539,7 +4531,7 @@
         <v>5</v>
       </c>
       <c r="D167" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
@@ -4553,7 +4545,7 @@
         <v>5</v>
       </c>
       <c r="D168" t="s">
-        <v>434</v>
+        <v>299</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
@@ -4567,7 +4559,7 @@
         <v>5</v>
       </c>
       <c r="D169" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
@@ -4581,119 +4573,119 @@
         <v>5</v>
       </c>
       <c r="D170" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
+      <c r="A171" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B171" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="B171" t="s">
-        <v>250</v>
-      </c>
-      <c r="C171" t="s">
+      <c r="C171" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D171" t="s">
-        <v>434</v>
+      <c r="D171" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A172" t="s">
-        <v>297</v>
-      </c>
-      <c r="B172" t="s">
-        <v>298</v>
-      </c>
-      <c r="C172" t="s">
+      <c r="A172" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B172" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="C172" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D172" t="s">
-        <v>434</v>
+      <c r="D172" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B173" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C173" t="s">
         <v>5</v>
       </c>
       <c r="D173" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A174" t="s">
+      <c r="A174" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B174" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C174" t="s">
+      <c r="C174" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D174" t="s">
-        <v>434</v>
+      <c r="D174" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A175" t="s">
+      <c r="A175" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B175" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C175" t="s">
+      <c r="C175" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D175" t="s">
-        <v>434</v>
+      <c r="D175" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A176" t="s">
+      <c r="A176" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B176" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="B176" t="s">
-        <v>234</v>
-      </c>
-      <c r="C176" t="s">
+      <c r="C176" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D176" t="s">
-        <v>434</v>
+      <c r="D176" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B177" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C177" t="s">
         <v>5</v>
       </c>
       <c r="D177" t="s">
-        <v>434</v>
+        <v>494</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
-        <v>489</v>
-      </c>
-      <c r="B178" t="s">
-        <v>490</v>
-      </c>
-      <c r="C178" t="s">
+      <c r="A178" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="B178" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="C178" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D178" t="s">
-        <v>434</v>
+      <c r="D178" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
@@ -4707,7 +4699,7 @@
         <v>5</v>
       </c>
       <c r="D179" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
@@ -4721,7 +4713,7 @@
         <v>5</v>
       </c>
       <c r="D180" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
@@ -4735,77 +4727,77 @@
         <v>5</v>
       </c>
       <c r="D181" t="s">
-        <v>496</v>
+        <v>432</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A182" t="s">
+      <c r="A182" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B182" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="B182" t="s">
-        <v>256</v>
-      </c>
-      <c r="C182" t="s">
+      <c r="C182" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D182" t="s">
-        <v>496</v>
+      <c r="D182" s="3" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
+        <v>265</v>
+      </c>
+      <c r="B183" t="s">
         <v>266</v>
-      </c>
-      <c r="B183" t="s">
-        <v>267</v>
       </c>
       <c r="C183" t="s">
         <v>5</v>
       </c>
       <c r="D183" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B184" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C184" t="s">
         <v>5</v>
       </c>
       <c r="D184" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B185" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C185" t="s">
         <v>5</v>
       </c>
       <c r="D185" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="B186" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="C186" t="s">
         <v>5</v>
       </c>
       <c r="D186" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.25">
@@ -4819,7 +4811,7 @@
         <v>81</v>
       </c>
       <c r="D187" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.25">
@@ -4833,287 +4825,287 @@
         <v>81</v>
       </c>
       <c r="D188" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
+        <v>216</v>
+      </c>
+      <c r="B189" t="s">
         <v>217</v>
-      </c>
-      <c r="B189" t="s">
-        <v>218</v>
       </c>
       <c r="C189" t="s">
         <v>81</v>
       </c>
       <c r="D189" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
+        <v>220</v>
+      </c>
+      <c r="B190" t="s">
         <v>221</v>
-      </c>
-      <c r="B190" t="s">
-        <v>222</v>
       </c>
       <c r="C190" t="s">
         <v>81</v>
       </c>
       <c r="D190" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
+        <v>267</v>
+      </c>
+      <c r="B191" t="s">
         <v>268</v>
-      </c>
-      <c r="B191" t="s">
-        <v>269</v>
       </c>
       <c r="C191" t="s">
         <v>81</v>
       </c>
       <c r="D191" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B192" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C192" t="s">
         <v>81</v>
       </c>
       <c r="D192" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B193" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C193" t="s">
         <v>81</v>
       </c>
       <c r="D193" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B194" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C194" t="s">
         <v>81</v>
       </c>
       <c r="D194" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B195" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C195" t="s">
         <v>81</v>
       </c>
       <c r="D195" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B196" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C196" t="s">
         <v>81</v>
       </c>
       <c r="D196" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B197" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C197" t="s">
         <v>81</v>
       </c>
       <c r="D197" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B198" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C198" t="s">
         <v>81</v>
       </c>
       <c r="D198" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B199" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C199" t="s">
         <v>81</v>
       </c>
       <c r="D199" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B200" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C200" t="s">
         <v>81</v>
       </c>
       <c r="D200" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B201" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C201" t="s">
         <v>81</v>
       </c>
       <c r="D201" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B202" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C202" t="s">
         <v>81</v>
       </c>
       <c r="D202" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B203" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="C203" t="s">
         <v>81</v>
       </c>
       <c r="D203" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B204" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C204" t="s">
         <v>81</v>
       </c>
       <c r="D204" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B205" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C205" t="s">
         <v>81</v>
       </c>
       <c r="D205" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B206" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C206" t="s">
         <v>81</v>
       </c>
       <c r="D206" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B207" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="C207" t="s">
         <v>81</v>
       </c>
       <c r="D207" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B208" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C208" t="s">
         <v>81</v>
       </c>
       <c r="D208" t="s">
-        <v>547</v>
+        <v>528</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
@@ -5127,7 +5119,7 @@
         <v>41</v>
       </c>
       <c r="D209" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
@@ -5141,7 +5133,7 @@
         <v>41</v>
       </c>
       <c r="D210" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
@@ -5155,7 +5147,7 @@
         <v>41</v>
       </c>
       <c r="D211" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
@@ -5169,231 +5161,231 @@
         <v>41</v>
       </c>
       <c r="D212" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
+        <v>205</v>
+      </c>
+      <c r="B213" t="s">
         <v>206</v>
-      </c>
-      <c r="B213" t="s">
-        <v>207</v>
       </c>
       <c r="C213" t="s">
         <v>41</v>
       </c>
       <c r="D213" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
+        <v>214</v>
+      </c>
+      <c r="B214" t="s">
         <v>215</v>
-      </c>
-      <c r="B214" t="s">
-        <v>216</v>
       </c>
       <c r="C214" t="s">
         <v>41</v>
       </c>
       <c r="D214" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
+        <v>256</v>
+      </c>
+      <c r="B215" t="s">
         <v>257</v>
-      </c>
-      <c r="B215" t="s">
-        <v>258</v>
       </c>
       <c r="C215" t="s">
         <v>41</v>
       </c>
       <c r="D215" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B216" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C216" t="s">
         <v>41</v>
       </c>
       <c r="D216" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B217" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C217" t="s">
         <v>41</v>
       </c>
       <c r="D217" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B218" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C218" t="s">
         <v>41</v>
       </c>
       <c r="D218" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B219" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C219" t="s">
         <v>41</v>
       </c>
       <c r="D219" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B220" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C220" t="s">
         <v>41</v>
       </c>
       <c r="D220" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B221" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C221" t="s">
         <v>41</v>
       </c>
       <c r="D221" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B222" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="C222" t="s">
         <v>41</v>
       </c>
       <c r="D222" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B223" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C223" t="s">
         <v>41</v>
       </c>
       <c r="D223" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B224" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C224" t="s">
         <v>41</v>
       </c>
       <c r="D224" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="B225" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C225" t="s">
         <v>41</v>
       </c>
       <c r="D225" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B226" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C226" t="s">
         <v>41</v>
       </c>
       <c r="D226" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B227" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C227" t="s">
         <v>41</v>
       </c>
       <c r="D227" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="B228" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="C228" t="s">
         <v>41</v>
       </c>
       <c r="D228" t="s">
-        <v>548</v>
+        <v>257</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
@@ -5407,7 +5399,7 @@
         <v>16</v>
       </c>
       <c r="D229" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
@@ -5421,7 +5413,7 @@
         <v>16</v>
       </c>
       <c r="D230" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
@@ -5435,7 +5427,7 @@
         <v>16</v>
       </c>
       <c r="D231" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
@@ -5449,7 +5441,7 @@
         <v>16</v>
       </c>
       <c r="D232" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
@@ -5463,7 +5455,7 @@
         <v>16</v>
       </c>
       <c r="D233" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
@@ -5477,189 +5469,189 @@
         <v>16</v>
       </c>
       <c r="D234" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
+        <v>189</v>
+      </c>
+      <c r="B235" t="s">
         <v>190</v>
-      </c>
-      <c r="B235" t="s">
-        <v>191</v>
       </c>
       <c r="C235" t="s">
         <v>16</v>
       </c>
       <c r="D235" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
+        <v>218</v>
+      </c>
+      <c r="B236" t="s">
         <v>219</v>
-      </c>
-      <c r="B236" t="s">
-        <v>220</v>
       </c>
       <c r="C236" t="s">
         <v>16</v>
       </c>
       <c r="D236" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
+        <v>240</v>
+      </c>
+      <c r="B237" t="s">
         <v>241</v>
-      </c>
-      <c r="B237" t="s">
-        <v>242</v>
       </c>
       <c r="C237" t="s">
         <v>16</v>
       </c>
       <c r="D237" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
+        <v>246</v>
+      </c>
+      <c r="B238" t="s">
         <v>247</v>
-      </c>
-      <c r="B238" t="s">
-        <v>248</v>
       </c>
       <c r="C238" t="s">
         <v>16</v>
       </c>
       <c r="D238" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
+        <v>269</v>
+      </c>
+      <c r="B239" t="s">
         <v>270</v>
-      </c>
-      <c r="B239" t="s">
-        <v>271</v>
       </c>
       <c r="C239" t="s">
         <v>16</v>
       </c>
       <c r="D239" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B240" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C240" t="s">
         <v>16</v>
       </c>
       <c r="D240" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B241" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C241" t="s">
         <v>16</v>
       </c>
       <c r="D241" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B242" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C242" t="s">
         <v>16</v>
       </c>
       <c r="D242" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B243" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="C243" t="s">
         <v>16</v>
       </c>
       <c r="D243" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="B244" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="C244" t="s">
         <v>16</v>
       </c>
       <c r="D244" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B245" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C245" t="s">
         <v>16</v>
       </c>
       <c r="D245" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="B246" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C246" t="s">
         <v>16</v>
       </c>
       <c r="D246" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B247" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C247" t="s">
         <v>16</v>
       </c>
       <c r="D247" t="s">
-        <v>549</v>
+        <v>247</v>
       </c>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
@@ -5678,10 +5670,10 @@
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
+        <v>195</v>
+      </c>
+      <c r="B249" t="s">
         <v>196</v>
-      </c>
-      <c r="B249" t="s">
-        <v>197</v>
       </c>
       <c r="C249" t="s">
         <v>149</v>
@@ -5692,10 +5684,10 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B250" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="C250" t="s">
         <v>149</v>
@@ -5706,10 +5698,10 @@
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B251" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="C251" t="s">
         <v>149</v>
@@ -5729,7 +5721,7 @@
         <v>58</v>
       </c>
       <c r="D252" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
@@ -5743,7 +5735,7 @@
         <v>58</v>
       </c>
       <c r="D253" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
@@ -5757,77 +5749,88 @@
         <v>58</v>
       </c>
       <c r="D254" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
+        <v>263</v>
+      </c>
+      <c r="B255" t="s">
         <v>264</v>
-      </c>
-      <c r="B255" t="s">
-        <v>265</v>
       </c>
       <c r="C255" t="s">
         <v>58</v>
       </c>
       <c r="D255" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
+        <v>209</v>
+      </c>
+      <c r="B256" t="s">
         <v>210</v>
       </c>
-      <c r="B256" t="s">
+      <c r="C256" t="s">
         <v>211</v>
       </c>
-      <c r="C256" t="s">
-        <v>212</v>
-      </c>
       <c r="D256" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
+        <v>252</v>
+      </c>
+      <c r="B257" t="s">
         <v>253</v>
       </c>
-      <c r="B257" t="s">
-        <v>254</v>
-      </c>
       <c r="C257" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D257" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B258" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C258" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D258" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B259" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C259" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D259" t="s">
-        <v>294</v>
+        <v>292</v>
+      </c>
+    </row>
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B260" t="s">
+        <v>545</v>
+      </c>
+      <c r="C260" t="s">
+        <v>2</v>
+      </c>
+      <c r="D260" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>